<commit_message>
feat(F-NAR-019): ATOM-AUT.RAN.001-03 Le pain d'Amir
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.RAN.001-03.xlsx
+++ b/stories/arbres/ATOM-AUT.RAN.001-03.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut livrer le pain chaud au bout du couloir, avec son doudou. La maison de cubes tombe sur le doudou. Il cherche, met cubes puis voitures dans la caisse. Le doudou apparaît sous les voitures. Ils goûtent.</t>
+          <t>Une clochette de vélo traverse la rue. Ting. Sur la planche, un éclat de farine brille. Amir veut livrer le pain tiède au bout du couloir, maintenant. La maison de cubes tombe sur le doudou. Il cherche d'un coup : trou, table, tout écarter. Rien. Il refuse de foncer, met les cubes dans la caisse. Les voitures barrent le couloir. Il retrouve l'éclat près des roues. Le doudou apparaît. Sur la croûte, l'éclat garde une trace blanche.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Au loin, une clochette de vélo. Ting. Papa a de la farine sur le tablier. Une baguette craque quand il la casse. L'odeur du pain chaud remplit la maison. Il est encore tout chaud. Oui, il craque. Le couloir est un peu frais. Le tapis du salon est épais. En ce moment, Amir est à genoux. Des cubes rouges et bleus attendent. Je fais la boulangerie, maman. Une maison pour le pain ? Oui, avec une porte. Amir pose un cube rouge. Puis un cube bleu. La maison grandit au milieu du tapis. Les cubes font un bruit sec. Ta maison a une porte ? Une petite porte, papa. Amir laisse un trou. C'est la porte de la boulangerie. Le doudou beige est assis contre le mur. Toi, tu attends le pain. Papa pose un morceau tiède près de la porte. Les voitures vont le livrer. Jusqu'au bout du couloir ? Oui, on le mange là-bas. Amir prend une petite voiture rouge. Les roues font un bruit léger. La voiture avance. Elle bute contre un cube. Un pan de la maison glisse. Des cubes tombent sur le doudou. Oh. La maison a bougé. Amir cherche le tissu beige. Où est mon doudou ? Derrière la porte de la boulangerie ? Amir regarde le trou. Seulement le pain tiède. Sous la table ? Il se penche. L'ombre est vide. Il est perdu. Les cubes sont encore tout autour. Je veux voir dessous. Amir prend un cube rouge. Il le pose dans la caisse en bois. Toc. Le bois sent un peu la forêt.</t>
+          <t>Une clochette de vélo traverse la rue, nette. Ting. Dans la maison, l'odeur de croûte répond. Papa a de la farine sur le tablier. Sur la planche, un éclat de farine brille. Il est blanc, papa. C'est un reste de la fournée. L'éclat de farine tient comme une petite lune. Le tapis du salon est épais, chaud. Le couloir, plus loin, reste un peu frais. Le pain est tiède, Amir. Je le veux au bout, maintenant. Au bout du couloir ? Oui, on le mange là-bas. En ce moment, Amir est à genoux. Des cubes rouges et bleus attendent sur le tapis. Je fais la boulangerie, maman. Une maison pour le pain ? Oui, avec une petite porte. Amir pose un cube rouge, puis un bleu. La maison grandit au milieu du tapis. Les cubes font un bruit sec. Ta maison a une porte ? Une petite porte, papa. Amir laisse un trou, bien net. C'est la porte de la boulangerie. Le doudou beige est assis contre le mur. Toi, tu attends le pain. Papa pose un morceau tiède près de la porte. Les voitures vont le livrer. Amir prend une petite voiture rouge. Les roues font un bruit léger sur le tapis. La voiture avance trop vite. Elle bute contre un cube. Un pan de la maison glisse. Des cubes tombent sur le doudou. Oh. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. La maison a bougé. Où est mon doudou ? Derrière la porte de la boulangerie ? Amir regarde le trou, d'un coup. Seulement le pain tiède. Sous la table ? Il se penche, trop vite. L'ombre est vide. Il est perdu. Amir veut tout écarter d'un seul geste. Les cubes glissent plus loin, plus nombreux. Ça ne veut pas. Ses épaules tombent un peu. Ça serre, dans son ventre. Maman se baisse à sa hauteur. Tu regardes sous les cubes ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Au loin, une clochette de vélo. Ting. Papa a de la farine sur le tablier. Une baguette craque quand il la casse. L'odeur du pain chaud remplit la maison. Il est encore tout chaud. Oui, il craque. Le couloir est un peu frais. Le tapis du salon est épais. En ce moment, Amir est à genoux. Des cubes rouges et bleus attendent. Je fais la boulangerie, maman. Une maison pour le pain ? Oui, avec une porte. Amir pose un cube rouge. Puis un cube bleu. La maison grandit au milieu du tapis. Les cubes font un bruit sec. Ta maison a une porte ? Une petite porte, papa. Amir laisse un trou. C'est la porte de la boulangerie. Le doudou beige est assis contre le mur. Toi, tu attends le pain. Papa pose un morceau tiède près de la porte. Les voitures vont le livrer. Jusqu'au bout du couloir ? Oui, on le mange là-bas. Amir prend une petite voiture rouge. Les roues font un bruit léger. La voiture avance. Elle bute contre un cube. Un pan de la maison glisse. Des cubes tombent sur le doudou. Oh. La maison a bougé. Amir cherche le tissu beige. Où est mon doudou ? Derrière la porte de la boulangerie ? Amir regarde le trou. Seulement le pain tiède. Sous la table ? Il se penche. L'ombre est vide. Il est perdu. Les cubes sont encore tout autour. Je veux voir dessous. Amir prend un cube rouge. Il le pose dans la caisse en bois. Toc. Le bois sent un peu la forêt.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une clochette de vélo traverse la rue, nette. Ting. Dans la maison, l'odeur de croûte répond. Papa a de la farine sur le tablier. Sur la planche, un &lt;emphasis level="moderate"&gt;éclat de farine&lt;/emphasis&gt; brille. Il est blanc, papa. C'est un reste de la fournée. L'éclat de farine tient comme une petite lune. Le tapis du salon est épais, chaud. Le couloir, plus loin, reste un peu frais. Le pain est tiède, Amir. Je le veux au bout, maintenant. Au bout du couloir ? Oui, on le mange là-bas. En ce moment, Amir est à genoux. Des cubes rouges et bleus attendent sur le tapis. Je fais la boulangerie, maman. Une maison pour le pain ? Oui, avec une petite porte. Amir pose un cube rouge, puis un bleu. La maison grandit au milieu du tapis. Les cubes font un bruit sec. Ta maison a une porte ? Une petite porte, papa. Amir laisse un trou, bien net. C'est la porte de la boulangerie. Le doudou beige est assis contre le mur. Toi, tu attends le pain. Papa pose un morceau tiède près de la porte. Les voitures vont le livrer. Amir prend une petite voiture rouge. Les roues font un bruit léger sur le tapis. La voiture avance trop vite. Elle bute contre un cube. Un pan de la maison glisse. Des cubes tombent sur le doudou. Oh. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. La maison a bougé. Où est mon doudou ? Derrière la porte de la boulangerie ? Amir regarde le trou, d'un coup. Seulement le pain tiède. Sous la table ? Il se penche, trop vite. L'ombre est vide. Il est perdu. Amir veut tout écarter d'un seul geste. Les cubes glissent plus loin, plus nombreux. Ça ne veut pas. Ses épaules tombent un peu. Ça serre, dans son ventre. Maman se baisse à sa hauteur. Tu regardes sous les cubes ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Kenzo joue aux cubes dans le salon. Les cubes font un bruit sec. Le tapis est doux. Maman dit : le jeu est fini. On va &lt;emphasis&gt;ranger&lt;/emphasis&gt;. Les jouets retournent dans la caisse. Kenzo prend les cubes, un par un. Il les met dans la caisse. La caisse est pleine. Maman dit : merci. Plus tard, Kenzo joue aux voitures dans le couloir. Les roues font un bruit léger. Maman dit : on range. Kenzo se souvient. Il prend les voitures. Il les met dans la caisse. Ranger, c'est mettre dans la caisse. Même leçon, autre lieu. Kenzo a rangé deux fois. [pause]</t>
+          <t>Une clochette de vélo traverse la rue, nette. Ting. Dans la maison, l'odeur de croûte répond. Papa a de la farine sur le tablier. Sur la planche, un &lt;emphasis&gt;éclat de farine&lt;/emphasis&gt; brille. Il est blanc, papa. C'est un reste de la fournée. L'éclat de farine tient comme une petite lune. Le tapis du salon est épais, chaud. Le couloir, plus loin, reste un peu frais. Le pain est tiède, Amir. Je le veux au bout, maintenant. Au bout du couloir ? Oui, on le mange là-bas. En ce moment, Amir est à genoux. Des cubes rouges et bleus attendent sur le tapis. Je fais la boulangerie, maman. Une maison pour le pain ? Oui, avec une petite porte. Amir pose un cube rouge, puis un bleu. La maison grandit au milieu du tapis. Les cubes font un bruit sec. Ta maison a une porte ? Une petite porte, papa. Amir laisse un trou, bien net. C'est la porte de la boulangerie. Le doudou beige est assis contre le mur. Toi, tu attends le pain. Papa pose un morceau tiède près de la porte. Les voitures vont le livrer. Amir prend une petite voiture rouge. Les roues font un bruit léger sur le tapis. La voiture avance trop vite. Elle bute contre un cube. Un pan de la maison glisse. Des cubes tombent sur le doudou. Oh. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. La maison a bougé. Où est mon doudou ? Derrière la porte de la boulangerie ? Amir regarde le trou, d'un coup. Seulement le pain tiède. Sous la table ? Il se penche, trop vite. L'ombre est vide. Il est perdu. Amir veut tout écarter d'un seul geste. Les cubes glissent plus loin, plus nombreux. Ça ne veut pas. Ses épaules tombent un peu. Ça serre, dans son ventre. Maman se baisse à sa hauteur. Tu regardes sous les cubes ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>ranger</t>
+          <t>éclat de farine</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,60 +1321,73 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_pain_au_bout_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Au loin, une clochette de vélo.
+          <t>narrateur|Une clochette de vélo traverse la rue, nette.
 narrateur|Ting.
+narrateur|Dans la maison, l'odeur de croûte répond.
 narrateur|Papa a de la farine sur le tablier.
-narrateur|Une baguette craque quand il la casse.
-narrateur|L'odeur du pain chaud remplit la maison.
-maman|Il est encore tout chaud.
-papa|Oui, il craque.
-narrateur|Le couloir est un peu frais.
-narrateur|Le tapis du salon est épais.
+narrateur|Sur la planche, un éclat de farine brille.
+enfant-m|Il est blanc, papa.
+papa|C'est un reste de la fournée.
+narrateur|L'éclat de farine tient comme une petite lune.
+narrateur|Le tapis du salon est épais, chaud.
+narrateur|Le couloir, plus loin, reste un peu frais.
+maman|Le pain est tiède, Amir.
+enfant-m|Je le veux au bout, maintenant.
+papa|Au bout du couloir ?
+enfant-m|Oui, on le mange là-bas.
 narrateur|En ce moment, Amir est à genoux.
-narrateur|Des cubes rouges et bleus attendent.
+narrateur|Des cubes rouges et bleus attendent sur le tapis.
 enfant-m|Je fais la boulangerie, maman.
 maman|Une maison pour le pain ?
-enfant-m|Oui, avec une porte.
-narrateur|Amir pose un cube rouge.
-narrateur|Puis un cube bleu.
+enfant-m|Oui, avec une petite porte.
+narrateur|Amir pose un cube rouge, puis un bleu.
 narrateur|La maison grandit au milieu du tapis.
 narrateur|Les cubes font un bruit sec.
 papa|Ta maison a une porte ?
 enfant-m|Une petite porte, papa.
-narrateur|Amir laisse un trou.
+narrateur|Amir laisse un trou, bien net.
 narrateur|C'est la porte de la boulangerie.
 narrateur|Le doudou beige est assis contre le mur.
 enfant-m|Toi, tu attends le pain.
 narrateur|Papa pose un morceau tiède près de la porte.
 enfant-m|Les voitures vont le livrer.
-papa|Jusqu'au bout du couloir ?
-enfant-m|Oui, on le mange là-bas.
 narrateur|Amir prend une petite voiture rouge.
-narrateur|Les roues font un bruit léger.
-narrateur|La voiture avance.
+narrateur|Les roues font un bruit léger sur le tapis.
+narrateur|La voiture avance trop vite.
 narrateur|Elle bute contre un cube.
 narrateur|Un pan de la maison glisse.
 narrateur|Des cubes tombent sur le doudou.
 enfant-m|Oh.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
 maman|La maison a bougé.
-narrateur|Amir cherche le tissu beige.
 enfant-m|Où est mon doudou ?
 papa|Derrière la porte de la boulangerie ?
-narrateur|Amir regarde le trou.
+narrateur|Amir regarde le trou, d'un coup.
 narrateur|Seulement le pain tiède.
 enfant-m|Sous la table ?
-narrateur|Il se penche.
+narrateur|Il se penche, trop vite.
 narrateur|L'ombre est vide.
 enfant-m|Il est perdu.
-maman|Les cubes sont encore tout autour.
-enfant-m|Je veux voir dessous.
-narrateur|Amir prend un cube rouge.
-narrateur|Il le pose dans la caisse en bois.
-narrateur|Toc.
-narrateur|Le bois sent un peu la forêt.</t>
+narrateur|Amir veut tout écarter d'un seul geste.
+narrateur|Les cubes glissent plus loin, plus nombreux.
+enfant-m|Ça ne veut pas.
+narrateur|Ses épaules tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Maman se baisse à sa hauteur.
+maman|Tu regardes sous les cubes ?</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>clochette,cubes,voiture</t>
         </is>
       </c>
     </row>
@@ -1406,12 +1419,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Amir cherche son doudou. Où est-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Amir cherche son &lt;emphasis level="moderate"&gt;doudou&lt;/emphasis&gt;. Où est-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Le jeu est fini. Que fait Kenzo ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Amir cherche son &lt;emphasis&gt;doudou&lt;/emphasis&gt;. Où est-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1474,7 +1487,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1482,10 +1495,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1500,34 +1513,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>doudou</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1536,23 +1553,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_doudou_est_sous_le_bazar; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1585,17 +1602,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Un cube bleu va dans la caisse. Toc. Amir écarte encore un mur. Tu regardes bien sous la maison ? Oui, maman. Le tapis reparaît, un peu. Pas de tissu beige. Peut-être plus loin, vers le couloir. Amir prend le morceau de pain. Il le pose sur la voiture rouge. On va au bout. Le couloir est un peu frais. D'autres petites voitures attendent. Une voiture bleue barre le chemin. Une jaune aussi. Elles cachent le sol. Amir glisse la bleue dans la caisse. Toc. Puis la jaune. Un bout de tissu dépasse près de la porte. Mon doudou ! Le doudou était sous les voitures. Il sent encore le tapis du salon. Amir le serre contre sa joue. Merci, tu l'as trouvé. Te voilà, petit. Il était sous les roues. Le bout du couloir est libre, maintenant.</t>
+          <t>Amir refuse d'écarter tout d'un coup. Il pose un genou sur le tapis. Un cube rouge va dans la caisse. Toc. Le bois sent un peu la forêt. Je le mets, maman. Tu regardes bien sous la maison ? Oui, maman. Un cube bleu rejoint le rouge. Le tapis reparaît, un peu. Pas de tissu beige. Peut-être plus loin, vers le couloir. Amir prend le morceau de pain. Il le pose sur la voiture rouge. On va au bout. Le couloir est un peu frais. D'autres petites voitures attendent. Une voiture bleue barre le chemin. Une jaune aussi. Elles cachent le sol. Amir veut les pousser d'un coup. Puis il s'arrête. Attends, je regarde. Amir refuse de foncer. Il écoute le couloir, un instant. Sur le tapis, un éclat de farine brille. Comme sur la planche ! Tu le vois, toi ? Oui, près des roues. Amir glisse la bleue dans la caisse. Toc. Puis la jaune. Un bout de tissu dépasse près de la porte. Mon doudou ! Le doudou était sous les voitures. Un éclat de farine tient sur son oreille. Amir le serre contre sa joue. Merci, tu l'as trouvé. Te voilà, petit. Il était sous les roues.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Un cube bleu va dans la caisse. Toc. Amir écarte encore un mur. Tu regardes bien sous la maison ? Oui, maman. Le tapis reparaît, un peu. Pas de tissu beige. Peut-être plus loin, vers le couloir. Amir prend le morceau de pain. Il le pose sur la voiture rouge. On va au bout. Le couloir est un peu frais. D'autres petites voitures attendent. Une voiture bleue barre le chemin. Une jaune aussi. Elles cachent le sol. Amir glisse la bleue dans la caisse. Toc. Puis la jaune. Un bout de tissu dépasse près de la porte. Mon doudou ! Le doudou était sous les voitures. Il sent encore le tapis du salon. Amir le serre contre sa joue. Merci, tu l'as trouvé. Te voilà, petit. Il était sous les roues. Le bout du couloir est libre, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir refuse d'écarter tout d'un coup. Il pose un genou sur le tapis. Un cube rouge va dans la caisse. Toc. Le bois sent un peu la forêt. Je le mets, maman. Tu regardes bien sous la maison ? Oui, maman. Un cube bleu rejoint le rouge. Le tapis reparaît, un peu. Pas de tissu beige. Peut-être plus loin, vers le couloir. Amir prend le morceau de pain. Il le pose sur la voiture rouge. On va au bout. Le couloir est un peu frais. D'autres petites voitures attendent. Une voiture bleue barre le chemin. Une jaune aussi. Elles cachent le sol. Amir veut les pousser d'un coup. Puis il s'arrête. Attends, je regarde. Amir refuse de foncer. Il écoute le couloir, un instant. Sur le tapis, un &lt;emphasis level="moderate"&gt;éclat de farine&lt;/emphasis&gt; brille. Comme sur la planche ! Tu le vois, toi ? Oui, près des roues. Amir glisse la bleue dans la caisse. Toc. Puis la jaune. Un bout de tissu dépasse près de la porte. Mon doudou ! Le doudou était sous les voitures. Un éclat de farine tient sur son oreille. Amir le serre contre sa joue. Merci, tu l'as trouvé. Te voilà, petit. Il était sous les roues.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Kenzo a rangé les cubes. Puis les voitures. Dans la &lt;emphasis&gt;caisse&lt;/emphasis&gt;, deux fois. [pause]</t>
+          <t>Amir refuse d'écarter tout d'un coup. Il pose un genou sur le tapis. Un cube rouge va dans la caisse. Toc. Le bois sent un peu la forêt. Je le mets, maman. Tu regardes bien sous la maison ? Oui, maman. Un cube bleu rejoint le rouge. Le tapis reparaît, un peu. Pas de tissu beige. Peut-être plus loin, vers le couloir. Amir prend le morceau de pain. Il le pose sur la voiture rouge. On va au bout. Le couloir est un peu frais. D'autres petites voitures attendent. Une voiture bleue barre le chemin. Une jaune aussi. Elles cachent le sol. Amir veut les pousser d'un coup. Puis il s'arrête. Attends, je regarde. Amir refuse de foncer. Il écoute le couloir, un instant. Sur le tapis, un &lt;emphasis&gt;éclat de farine&lt;/emphasis&gt; brille. Comme sur la planche ! Tu le vois, toi ? Oui, près des roues. Amir glisse la bleue dans la caisse. Toc. Puis la jaune. Un bout de tissu dépasse près de la porte. Mon doudou ! Le doudou était sous les voitures. Un éclat de farine tient sur son oreille. Amir le serre contre sa joue. Merci, tu l'as trouvé. Te voilà, petit. Il était sous les roues. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1642,7 +1659,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1650,10 +1667,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1676,30 +1693,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>caisse</t>
+          <t>éclat de farine</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1708,10 +1725,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1724,16 +1741,20 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_retrouve_l_eclat; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Un cube bleu va dans la caisse.
+          <t>narrateur|Amir refuse d'écarter tout d'un coup.
+narrateur|Il pose un genou sur le tapis.
+narrateur|Un cube rouge va dans la caisse.
 narrateur|Toc.
-narrateur|Amir écarte encore un mur.
+narrateur|Le bois sent un peu la forêt.
+enfant-m|Je le mets, maman.
 maman|Tu regardes bien sous la maison ?
 enfant-m|Oui, maman.
+narrateur|Un cube bleu rejoint le rouge.
 narrateur|Le tapis reparaît, un peu.
 narrateur|Pas de tissu beige.
 papa|Peut-être plus loin, vers le couloir.
@@ -1745,18 +1766,31 @@
 narrateur|Une voiture bleue barre le chemin.
 narrateur|Une jaune aussi.
 enfant-m|Elles cachent le sol.
+narrateur|Amir veut les pousser d'un coup.
+narrateur|Puis il s'arrête.
+enfant-m|Attends, je regarde.
+narrateur|Amir refuse de foncer.
+narrateur|Il écoute le couloir, un instant.
+narrateur|Sur le tapis, un éclat de farine brille.
+enfant-m|Comme sur la planche !
+papa|Tu le vois, toi ?
+enfant-m|Oui, près des roues.
 narrateur|Amir glisse la bleue dans la caisse.
 narrateur|Toc.
 narrateur|Puis la jaune.
 narrateur|Un bout de tissu dépasse près de la porte.
 enfant-m|Mon doudou !
 narrateur|Le doudou était sous les voitures.
-narrateur|Il sent encore le tapis du salon.
+narrateur|Un éclat de farine tient sur son oreille.
 narrateur|Amir le serre contre sa joue.
 papa|Merci, tu l'as trouvé.
 maman|Te voilà, petit.
-enfant-m|Il était sous les roues.
-narrateur|Le bout du couloir est libre, maintenant.</t>
+enfant-m|Il était sous les roues.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>caisse,voitures</t>
         </is>
       </c>
     </row>
@@ -1783,17 +1817,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>L'horloge fait tic-tac, tout doux. Amir s'assoit au bout du couloir. Le doudou est sur ses genoux. Papa lui tend le morceau de pain. La croûte craque encore. Il est chaud. On le mange ici, comme prévu. Tu veux une petite miette pour lui ? Une toute petite. Amir pose une miette sur le tissu. Le doudou reste bien droit. L'odeur du pain remplit le couloir. On est bien, ici. La voiture a fini la course. Oui, jusqu'au bout.</t>
+          <t>Amir s'assoit au bout du couloir. Le doudou est sur ses genoux. Papa lui tend le morceau de pain. La croûte craque sous les dents. Il est chaud. On le mange ici, comme prévu. Tu veux une petite miette pour lui ? Une toute petite. Amir pose une miette sur le tissu. Le doudou reste bien droit. L'odeur du pain remplit le couloir. On est bien, ici. La voiture a fini la course. Oui, jusqu'au bout. Sur la croûte, un éclat de farine brille. Comme sur la planche, papa. Au loin, la clochette de vélo reprend. Ting.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>L'horloge fait tic-tac, tout doux. Amir s'assoit au bout du couloir. Le doudou est sur ses genoux. Papa lui tend le morceau de pain. La croûte craque encore. Il est chaud. On le mange ici, comme prévu. Tu veux une petite miette pour lui ? Une toute petite. Amir pose une miette sur le tissu. Le doudou reste bien droit. L'odeur du pain remplit le couloir. On est bien, ici. La voiture a fini la course. Oui, jusqu'au bout.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir s'assoit au bout du couloir. Le doudou est sur ses genoux. Papa lui tend le morceau de &lt;emphasis level="moderate"&gt;pain&lt;/emphasis&gt;. La croûte craque sous les dents. Il est chaud. On le mange ici, comme prévu. Tu veux une petite miette pour lui ? Une toute petite. Amir pose une miette sur le tissu. Le doudou reste bien droit. L'odeur du pain remplit le couloir. On est bien, ici. La voiture a fini la course. Oui, jusqu'au bout. Sur la croûte, un éclat de farine brille. Comme sur la planche, papa. Au loin, la clochette de vélo reprend. Ting.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;caisse&lt;/emphasis&gt; est fermée. Maman sourit. [pause]</t>
+          <t>Amir s'assoit au bout du couloir. Le doudou est sur ses genoux. Papa lui tend le morceau de &lt;emphasis&gt;pain&lt;/emphasis&gt;. La croûte craque sous les dents. Il est chaud. On le mange ici, comme prévu. Tu veux une petite miette pour lui ? Une toute petite. Amir pose une miette sur le tissu. Le doudou reste bien droit. L'odeur du pain remplit le couloir. On est bien, ici. La voiture a fini la course. Oui, jusqu'au bout. Sur la croûte, un éclat de farine brille. Comme sur la planche, papa. Au loin, la clochette de vélo reprend. Ting. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1840,7 +1874,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1848,10 +1882,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1874,30 +1908,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>caisse</t>
+          <t>pain</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1906,10 +1940,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1920,14 +1954,17 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=refermer_le_désir; emotion=fierté_calme et chaleur; intensite=2; destinataire=enfant; sous_texte=le_pain_arrive_au_bout; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|L'horloge fait tic-tac, tout doux.
-narrateur|Amir s'assoit au bout du couloir.
+          <t>narrateur|Amir s'assoit au bout du couloir.
 narrateur|Le doudou est sur ses genoux.
 narrateur|Papa lui tend le morceau de pain.
-narrateur|La croûte craque encore.
+narrateur|La croûte craque sous les dents.
 enfant-m|Il est chaud.
 maman|On le mange ici, comme prévu.
 papa|Tu veux une petite miette pour lui ?
@@ -1937,7 +1974,16 @@
 narrateur|L'odeur du pain remplit le couloir.
 maman|On est bien, ici.
 enfant-m|La voiture a fini la course.
-papa|Oui, jusqu'au bout.</t>
+papa|Oui, jusqu'au bout.
+narrateur|Sur la croûte, un éclat de farine brille.
+enfant-m|Comme sur la planche, papa.
+narrateur|Au loin, la clochette de vélo reprend.
+narrateur|Ting.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>pain,couloir</t>
         </is>
       </c>
     </row>
@@ -1964,17 +2010,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a du pain. Toi aussi. Bravo, tu l'as retrouvé. La farine reste un peu sur le tablier. Le couloir sent encore la croûte chaude.</t>
+          <t>Le doudou a du pain. Toi aussi. La farine reste un peu sur le tablier. Le couloir sent la croûte chaude. La chaleur touche les joues d'Amir. Sur le pain, l'éclat de farine garde une trace blanche.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a du pain. Toi aussi. Bravo, tu l'as retrouvé. La farine reste un peu sur le tablier. Le couloir sent encore la croûte chaude.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou a du pain. Toi aussi. La farine reste un peu sur le tablier. Le couloir sent la croûte chaude. La chaleur touche les joues d'Amir. Sur le pain, l'&lt;emphasis level="moderate"&gt;éclat de farine&lt;/emphasis&gt; garde une trace blanche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou a du pain. Toi aussi. La farine reste un peu sur le tablier. Le couloir sent la croûte chaude. La chaleur touche les joues d'Amir. Sur le pain, l'&lt;emphasis&gt;éclat de farine&lt;/emphasis&gt; garde une trace blanche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2021,18 +2067,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2041,12 +2087,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2055,17 +2101,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de farine</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2074,11 +2124,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2087,28 +2137,38 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_la_planche_est_sur_la_croute; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
           <t>enfant-m|Le doudou a du pain.
 maman|Toi aussi.
-papa|Bravo, tu l'as retrouvé.
 narrateur|La farine reste un peu sur le tablier.
-narrateur|Le couloir sent encore la croûte chaude.</t>
+narrateur|Le couloir sent la croûte chaude.
+narrateur|La chaleur touche les joues d'Amir.
+narrateur|Sur le pain, l'éclat de farine garde une trace blanche.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>farine,pain</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2193,6 +2253,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>